<commit_message>
sdt adaptor fixed, BOM files works successfully, new cdf of sdt adaptor added
</commit_message>
<xml_diff>
--- a/timestamps_component/plot_timestamps/timestamps_results.xlsx
+++ b/timestamps_component/plot_timestamps/timestamps_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aabishek\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67406F7-63CD-4B77-84BB-140DB6015009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81769283-4A80-4DE0-8FDE-C2DF0BC06385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="45" windowWidth="29040" windowHeight="15720" xr2:uid="{76156820-5E03-4ABF-8EE4-B5EF3E2966AB}"/>
   </bookViews>
@@ -534,7 +534,7 @@
         <v>3.5630999999999999</v>
       </c>
       <c r="K2">
-        <v>1.15E-2</v>
+        <v>1.3299999999999999E-2</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -571,7 +571,7 @@
         <v>3.3435000000000001</v>
       </c>
       <c r="K3">
-        <v>8.5000000000000006E-3</v>
+        <v>1.2699999999999999E-2</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -608,7 +608,7 @@
         <v>3.2399</v>
       </c>
       <c r="K4">
-        <v>7.9000000000000008E-3</v>
+        <v>1.2500000000000001E-2</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -645,7 +645,7 @@
         <v>3.2507000000000001</v>
       </c>
       <c r="K5">
-        <v>7.4999999999999997E-3</v>
+        <v>1.2E-2</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -682,7 +682,7 @@
         <v>1.9626999999999999</v>
       </c>
       <c r="K6">
-        <v>8.3000000000000001E-3</v>
+        <v>1.32E-2</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -719,7 +719,7 @@
         <v>3.4836999999999998</v>
       </c>
       <c r="K7">
-        <v>7.4000000000000003E-3</v>
+        <v>1.24E-2</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -756,7 +756,7 @@
         <v>3.4660000000000002</v>
       </c>
       <c r="K8">
-        <v>7.6E-3</v>
+        <v>1.17E-2</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -793,7 +793,7 @@
         <v>3.2873000000000001</v>
       </c>
       <c r="K9">
-        <v>7.4000000000000003E-3</v>
+        <v>1.21E-2</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -830,7 +830,7 @@
         <v>3.2296</v>
       </c>
       <c r="K10">
-        <v>8.0000000000000002E-3</v>
+        <v>1.2200000000000001E-2</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -867,7 +867,7 @@
         <v>1.7822</v>
       </c>
       <c r="K11">
-        <v>7.7999999999999996E-3</v>
+        <v>1.21E-2</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -904,7 +904,7 @@
         <v>1.6970000000000001</v>
       </c>
       <c r="K12">
-        <v>8.2000000000000007E-3</v>
+        <v>1.18E-2</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
@@ -941,7 +941,7 @@
         <v>1.7201</v>
       </c>
       <c r="K13">
-        <v>7.6E-3</v>
+        <v>1.49E-2</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -978,7 +978,7 @@
         <v>3.2473000000000001</v>
       </c>
       <c r="K14">
-        <v>7.4999999999999997E-3</v>
+        <v>1.2E-2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -1015,7 +1015,7 @@
         <v>1.7330000000000001</v>
       </c>
       <c r="K15">
-        <v>7.6E-3</v>
+        <v>1.1900000000000001E-2</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
@@ -1052,7 +1052,7 @@
         <v>1.7214</v>
       </c>
       <c r="K16">
-        <v>8.3000000000000001E-3</v>
+        <v>1.29E-2</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
@@ -1089,7 +1089,7 @@
         <v>3.2410999999999999</v>
       </c>
       <c r="K17">
-        <v>8.2000000000000007E-3</v>
+        <v>1.21E-2</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -1126,7 +1126,7 @@
         <v>1.7211000000000001</v>
       </c>
       <c r="K18">
-        <v>8.3000000000000001E-3</v>
+        <v>1.18E-2</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
@@ -1163,7 +1163,7 @@
         <v>3.2484000000000002</v>
       </c>
       <c r="K19">
-        <v>7.6E-3</v>
+        <v>1.35E-2</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
@@ -1200,7 +1200,7 @@
         <v>3.2507000000000001</v>
       </c>
       <c r="K20">
-        <v>8.0999999999999996E-3</v>
+        <v>1.2699999999999999E-2</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
@@ -1237,7 +1237,7 @@
         <v>1.7330000000000001</v>
       </c>
       <c r="K21">
-        <v>8.8999999999999999E-3</v>
+        <v>1.46E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>